<commit_message>
Sync product catalog from September 2026 workbook (v8, 14 new products)
Regenerate data/products_db.json from the new Data_base_products.xlsx:
106 products (was 92). Added the Daurikus 50g and Oscietra Gold 50g
tins, the Signature range (Daurikus 30/50/250/500g, Baenki 1.8kg,
En-K 15g/250g/125g) and three empty-tin marketing items. No products
removed or changed.

Bump the boot maintenance script to v8 so hosted databases pick up the
new catalog on next deploy (catalog refresh only — consumption, stock,
forecasts and accounts are untouched).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018W7NxFXoeXGaFsJkP1KqtT
</commit_message>
<xml_diff>
--- a/data/Data_base_products.xlsx
+++ b/data/Data_base_products.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabien\Desktop\Kaviari Cellar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1642F5D7-4582-4822-97FB-130A530D86DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E680A9F5-A465-4716-86D7-BB8CB3DB35CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C1C395D8-19D5-4EE8-9504-7413A88F6FBD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C1C395D8-19D5-4EE8-9504-7413A88F6FBD}"/>
   </bookViews>
   <sheets>
     <sheet name="description" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="130">
   <si>
     <t>PR Code</t>
   </si>
@@ -392,6 +392,48 @@
   </si>
   <si>
     <t>Kaviari Baenki caviar 125 g/Tin</t>
+  </si>
+  <si>
+    <t>Empty Tin Bottom 50 g</t>
+  </si>
+  <si>
+    <t>Empty Tin Top 50 g</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Daurikus (50 g/tin)</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Oscietra Gold (50 g/tin)</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Daurikus (30g/tin)</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Daurikus (50g/tin) Signature</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Baenki (1.8kg/tin) Signature</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Baenki En-k (15g/tin) Signature</t>
+  </si>
+  <si>
+    <t>Kaviar Caviar Baenki (250g/tin) Signature</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Baenki (125g/tin) Signature</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Daurikus (250g/Tin) Signature</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Daurikus (500g/tin) Signature</t>
+  </si>
+  <si>
+    <t>Empty Tin Lid 30/50 g</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Daurikus (30g/tin) Signature</t>
   </si>
 </sst>
 </file>
@@ -425,7 +467,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -436,6 +478,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF156082"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -479,7 +527,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -490,17 +538,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,6 +565,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -835,9 +888,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}">
-  <dimension ref="A3:G95"/>
+  <dimension ref="A3:G109"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="9.140625" style="9"/>
     <col min="2" max="2" width="68.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
@@ -2354,25 +2408,25 @@
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" s="8">
+      <c r="A78" s="6">
         <v>8993</v>
       </c>
-      <c r="B78" s="9" t="s">
+      <c r="B78" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="C78" s="9" t="s">
+      <c r="C78" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D78" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="E78" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="F78" s="10">
+      <c r="D78" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E78" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="F78" s="8">
         <v>12</v>
       </c>
-      <c r="G78" s="10" t="s">
+      <c r="G78" s="8" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2571,10 +2625,10 @@
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A89" s="6">
+      <c r="A89" s="1">
         <v>9573</v>
       </c>
-      <c r="B89" s="7" t="s">
+      <c r="B89" s="2" t="s">
         <v>109</v>
       </c>
       <c r="C89" s="2" t="s">
@@ -2594,10 +2648,10 @@
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A90" s="6">
+      <c r="A90" s="1">
         <v>3341</v>
       </c>
-      <c r="B90" s="7" t="s">
+      <c r="B90" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C90" s="2" t="s">
@@ -2632,7 +2686,7 @@
       <c r="E91" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F91" s="11">
+      <c r="F91" s="3">
         <v>1</v>
       </c>
       <c r="G91" s="3" t="s">
@@ -2655,7 +2709,7 @@
       <c r="E92" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F92" s="11">
+      <c r="F92" s="3">
         <v>1</v>
       </c>
       <c r="G92" s="3" t="s">
@@ -2678,7 +2732,7 @@
       <c r="E93" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F93" s="11">
+      <c r="F93" s="3">
         <v>2</v>
       </c>
       <c r="G93" s="3" t="s">
@@ -2701,7 +2755,7 @@
       <c r="E94" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F94" s="11">
+      <c r="F94" s="3">
         <v>5</v>
       </c>
       <c r="G94" s="3" t="s">
@@ -2724,12 +2778,316 @@
       <c r="E95" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F95" s="11">
+      <c r="F95" s="3">
         <v>12</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>88</v>
       </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A96" s="10">
+        <v>9628</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C96" s="11"/>
+      <c r="D96" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E96" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F96" s="11"/>
+      <c r="G96" s="11"/>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A97" s="10">
+        <v>9629</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C97" s="11"/>
+      <c r="D97" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E97" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F97" s="11"/>
+      <c r="G97" s="11"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A98" s="10">
+        <v>9631</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C98" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D98" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E98" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F98" s="11">
+        <v>24</v>
+      </c>
+      <c r="G98" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A99" s="10">
+        <v>9632</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C99" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D99" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E99" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F99" s="11">
+        <v>24</v>
+      </c>
+      <c r="G99" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A100" s="10">
+        <v>9648</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C100" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D100" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E100" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F100" s="11">
+        <v>24</v>
+      </c>
+      <c r="G100" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A101" s="10">
+        <v>9649</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C101" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D101" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E101" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F101" s="11">
+        <v>24</v>
+      </c>
+      <c r="G101" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A102" s="10">
+        <v>9650</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C102" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D102" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E102" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F102" s="11">
+        <v>24</v>
+      </c>
+      <c r="G102" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A103" s="10">
+        <v>9651</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C103" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D103" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E103" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F103" s="11">
+        <v>1</v>
+      </c>
+      <c r="G103" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A104" s="10">
+        <v>9652</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C104" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D104" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E104" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F104" s="11">
+        <v>10</v>
+      </c>
+      <c r="G104" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" s="10">
+        <v>9653</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C105" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D105" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E105" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F105" s="11">
+        <v>5</v>
+      </c>
+      <c r="G105" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A106" s="10">
+        <v>9654</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C106" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="D106" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E106" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F106" s="11">
+        <v>12</v>
+      </c>
+      <c r="G106" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A107" s="10">
+        <v>9655</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C107" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D107" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E107" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F107" s="11">
+        <v>5</v>
+      </c>
+      <c r="G107" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A108" s="10">
+        <v>9656</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C108" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D108" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E108" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F108" s="11">
+        <v>2</v>
+      </c>
+      <c r="G108" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A109" s="10">
+        <v>9657</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C109" s="11"/>
+      <c r="D109" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E109" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="F109" s="11"/>
+      <c r="G109" s="11"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:E95" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}"/>
@@ -2739,7 +3097,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D728A83-21A1-4AAF-B2FC-CCC59733812F}">
-  <dimension ref="A3:H95"/>
+  <dimension ref="A3:H109"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="68.140625" bestFit="1" customWidth="1"/>
@@ -4713,7 +5071,7 @@
       <c r="G89" s="3">
         <v>1.8</v>
       </c>
-      <c r="H89" s="12">
+      <c r="H89" s="5">
         <f>G89*F89</f>
         <v>945</v>
       </c>
@@ -4740,7 +5098,7 @@
       <c r="G90" s="3">
         <v>1</v>
       </c>
-      <c r="H90" s="12">
+      <c r="H90" s="5">
         <f t="shared" ref="H90:H95" si="5">G90*F90</f>
         <v>525</v>
       </c>
@@ -4767,7 +5125,7 @@
       <c r="G91" s="3">
         <v>0.5</v>
       </c>
-      <c r="H91" s="12">
+      <c r="H91" s="5">
         <f t="shared" si="5"/>
         <v>262.5</v>
       </c>
@@ -4794,7 +5152,7 @@
       <c r="G92" s="3">
         <v>0.25</v>
       </c>
-      <c r="H92" s="12">
+      <c r="H92" s="5">
         <f t="shared" si="5"/>
         <v>131.25</v>
       </c>
@@ -4821,16 +5179,16 @@
       <c r="G93" s="3">
         <v>0.125</v>
       </c>
-      <c r="H93" s="12">
+      <c r="H93" s="5">
         <f t="shared" si="5"/>
         <v>65.625</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A94" s="6">
+      <c r="A94" s="1">
         <v>9573</v>
       </c>
-      <c r="B94" s="7" t="s">
+      <c r="B94" s="2" t="s">
         <v>109</v>
       </c>
       <c r="C94" s="2" t="s">
@@ -4842,22 +5200,22 @@
       <c r="E94" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F94" s="12">
+      <c r="F94" s="5">
         <v>785</v>
       </c>
-      <c r="G94" s="11">
+      <c r="G94" s="3">
         <v>0.05</v>
       </c>
-      <c r="H94" s="12">
+      <c r="H94" s="5">
         <f t="shared" si="5"/>
         <v>39.25</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A95" s="6">
+      <c r="A95" s="1">
         <v>3341</v>
       </c>
-      <c r="B95" s="7" t="s">
+      <c r="B95" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C95" s="2" t="s">
@@ -4869,16 +5227,367 @@
       <c r="E95" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F95" s="12">
+      <c r="F95" s="5">
         <v>785</v>
       </c>
-      <c r="G95" s="11">
+      <c r="G95" s="3">
         <v>0.03</v>
       </c>
-      <c r="H95" s="12">
+      <c r="H95" s="5">
         <f t="shared" si="5"/>
         <v>23.55</v>
       </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" s="10">
+        <v>9628</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C96" s="2"/>
+      <c r="D96" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E96" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F96" s="5"/>
+      <c r="G96" s="3"/>
+      <c r="H96" s="5"/>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97" s="10">
+        <v>9629</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C97" s="2"/>
+      <c r="D97" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E97" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F97" s="5"/>
+      <c r="G97" s="3"/>
+      <c r="H97" s="5"/>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" s="10">
+        <v>9631</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E98" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F98" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G98" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H98" s="5">
+        <f>F98*G98</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" s="10">
+        <v>9632</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D99" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E99" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F99" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G99" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H99" s="5">
+        <f>F99*G99</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100" s="10">
+        <v>9648</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D100" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E100" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F100" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G100" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H100" s="5">
+        <f>F100*G100</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101" s="10">
+        <v>9649</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E101" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F101" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G101" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H101" s="5">
+        <f>F101*G101</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A102" s="10">
+        <v>9650</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D102" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E102" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F102" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G102" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H102" s="5">
+        <f>F102*G102</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103" s="10">
+        <v>9651</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C103" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E103" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F103" s="5">
+        <v>525</v>
+      </c>
+      <c r="G103" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="H103" s="5">
+        <f>F103*G103</f>
+        <v>945</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104" s="10">
+        <v>9652</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C104" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F104" s="5">
+        <v>525</v>
+      </c>
+      <c r="G104" s="3">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="H104" s="5">
+        <f>F104*G104</f>
+        <v>7.875</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105" s="10">
+        <v>9653</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F105" s="5">
+        <v>525</v>
+      </c>
+      <c r="G105" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="H105" s="5">
+        <f>F105*G105</f>
+        <v>131.25</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106" s="10">
+        <v>9654</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F106" s="5">
+        <v>525</v>
+      </c>
+      <c r="G106" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="H106" s="5">
+        <f>F106*G106</f>
+        <v>65.625</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107" s="10">
+        <v>9655</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C107" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F107" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G107" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="H107" s="5">
+        <f>F107*G107</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108" s="10">
+        <v>9656</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="C108" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F108" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G108" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H108" s="5">
+        <f>F108*G108</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109" s="10">
+        <v>9657</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C109" s="2"/>
+      <c r="D109" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E109" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F109" s="5"/>
+      <c r="G109" s="3"/>
+      <c r="H109" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:H88" xr:uid="{5D728A83-21A1-4AAF-B2FC-CCC59733812F}"/>

</xml_diff>

<commit_message>
Sync product catalog from 12 Sep 2026 workbook (v11, 2 new products)
Regenerate data/products_db.json from the new Data_base_products.xlsx:
108 products (was 106). Added the unpasteurized Kristal 125g (3112)
and the Daurikus 125g Signature (9647); the Baeri Royal 50g (8559)
gains its grams-per-tin, now read from the Cost sheet's Weight/Tin
column when present. Boot maintenance v11 re-syncs hosted databases
on deploy — consumption, customer sales, forecasts and accounts are
untouched.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018W7NxFXoeXGaFsJkP1KqtT
</commit_message>
<xml_diff>
--- a/data/Data_base_products.xlsx
+++ b/data/Data_base_products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabien\Desktop\Kaviari Cellar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E680A9F5-A465-4716-86D7-BB8CB3DB35CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D6293EA-E395-41E4-9EEB-52D73A43892C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C1C395D8-19D5-4EE8-9504-7413A88F6FBD}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Cost!$A$3:$H$88</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">description!$A$3:$E$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">description!$A$3:$E$110</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="132">
   <si>
     <t>PR Code</t>
   </si>
@@ -434,6 +434,12 @@
   </si>
   <si>
     <t>Kaviari Caviar Daurikus (30g/tin) Signature</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Kristal (125 g/tin)[unpasteurized]</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Daurikus (125g/tin) Signature</t>
   </si>
 </sst>
 </file>
@@ -527,7 +533,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -550,6 +556,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -565,10 +580,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -888,7 +899,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}">
-  <dimension ref="A3:G109"/>
+  <dimension ref="A3:G111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="9"/>
@@ -2792,15 +2803,15 @@
       <c r="B96" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C96" s="11"/>
-      <c r="D96" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E96" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="F96" s="11"/>
-      <c r="G96" s="11"/>
+      <c r="C96" s="13"/>
+      <c r="D96" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="E96" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F96" s="13"/>
+      <c r="G96" s="13"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A97" s="10">
@@ -2809,15 +2820,15 @@
       <c r="B97" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C97" s="11"/>
-      <c r="D97" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E97" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="F97" s="11"/>
-      <c r="G97" s="11"/>
+      <c r="C97" s="13"/>
+      <c r="D97" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="E97" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F97" s="13"/>
+      <c r="G97" s="13"/>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A98" s="10">
@@ -2826,19 +2837,19 @@
       <c r="B98" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="C98" s="11" t="s">
+      <c r="C98" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D98" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E98" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F98" s="11">
+      <c r="D98" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E98" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F98" s="3">
         <v>24</v>
       </c>
-      <c r="G98" s="11" t="s">
+      <c r="G98" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2849,19 +2860,19 @@
       <c r="B99" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C99" s="11" t="s">
+      <c r="C99" s="13" t="s">
         <v>100</v>
       </c>
-      <c r="D99" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E99" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F99" s="11">
+      <c r="D99" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="E99" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="F99" s="13">
         <v>24</v>
       </c>
-      <c r="G99" s="11" t="s">
+      <c r="G99" s="13" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2872,19 +2883,19 @@
       <c r="B100" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C100" s="11" t="s">
+      <c r="C100" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D100" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E100" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F100" s="11">
+      <c r="D100" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E100" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F100" s="3">
         <v>24</v>
       </c>
-      <c r="G100" s="11" t="s">
+      <c r="G100" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2895,19 +2906,19 @@
       <c r="B101" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C101" s="11" t="s">
+      <c r="C101" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D101" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E101" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F101" s="11">
+      <c r="D101" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E101" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F101" s="3">
         <v>24</v>
       </c>
-      <c r="G101" s="11" t="s">
+      <c r="G101" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2918,19 +2929,19 @@
       <c r="B102" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C102" s="11" t="s">
+      <c r="C102" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D102" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E102" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F102" s="11">
+      <c r="D102" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E102" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F102" s="3">
         <v>24</v>
       </c>
-      <c r="G102" s="11" t="s">
+      <c r="G102" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2941,19 +2952,19 @@
       <c r="B103" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="C103" s="11" t="s">
+      <c r="C103" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D103" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E103" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F103" s="11">
+      <c r="D103" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E103" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F103" s="3">
         <v>1</v>
       </c>
-      <c r="G103" s="11" t="s">
+      <c r="G103" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2964,19 +2975,19 @@
       <c r="B104" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C104" s="11" t="s">
+      <c r="C104" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D104" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E104" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F104" s="11">
+      <c r="D104" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F104" s="3">
         <v>10</v>
       </c>
-      <c r="G104" s="11" t="s">
+      <c r="G104" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2987,19 +2998,19 @@
       <c r="B105" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C105" s="11" t="s">
+      <c r="C105" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D105" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E105" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F105" s="11">
+      <c r="D105" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E105" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F105" s="3">
         <v>5</v>
       </c>
-      <c r="G105" s="11" t="s">
+      <c r="G105" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -3010,19 +3021,19 @@
       <c r="B106" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="C106" s="11" t="s">
+      <c r="C106" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D106" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E106" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F106" s="11">
+      <c r="D106" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E106" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F106" s="3">
         <v>12</v>
       </c>
-      <c r="G106" s="11" t="s">
+      <c r="G106" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -3033,19 +3044,19 @@
       <c r="B107" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C107" s="11" t="s">
+      <c r="C107" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D107" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E107" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F107" s="11">
+      <c r="D107" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E107" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F107" s="3">
         <v>5</v>
       </c>
-      <c r="G107" s="11" t="s">
+      <c r="G107" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -3056,19 +3067,19 @@
       <c r="B108" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C108" s="11" t="s">
+      <c r="C108" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D108" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="E108" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="F108" s="11">
+      <c r="D108" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E108" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F108" s="3">
         <v>2</v>
       </c>
-      <c r="G108" s="11" t="s">
+      <c r="G108" s="3" t="s">
         <v>88</v>
       </c>
     </row>
@@ -3079,25 +3090,71 @@
       <c r="B109" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="C109" s="11"/>
-      <c r="D109" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E109" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="F109" s="11"/>
-      <c r="G109" s="11"/>
+      <c r="C109" s="13"/>
+      <c r="D109" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="E109" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="F109" s="13"/>
+      <c r="G109" s="13"/>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A110" s="14">
+        <v>3112</v>
+      </c>
+      <c r="B110" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C110" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D110" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E110" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F110" s="11">
+        <v>12</v>
+      </c>
+      <c r="G110" s="11" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A111" s="14">
+        <v>9647</v>
+      </c>
+      <c r="B111" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C111" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D111" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E111" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F111" s="11">
+        <v>12</v>
+      </c>
+      <c r="G111" s="11" t="s">
+        <v>88</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E95" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}"/>
+  <autoFilter ref="A3:E110" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D728A83-21A1-4AAF-B2FC-CCC59733812F}">
-  <dimension ref="A3:H109"/>
+  <dimension ref="A3:H111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="68.140625" bestFit="1" customWidth="1"/>
@@ -5297,7 +5354,7 @@
         <v>0.05</v>
       </c>
       <c r="H98" s="5">
-        <f>F98*G98</f>
+        <f t="shared" ref="H98:H111" si="6">F98*G98</f>
         <v>60</v>
       </c>
     </row>
@@ -5324,7 +5381,7 @@
         <v>0.05</v>
       </c>
       <c r="H99" s="5">
-        <f>F99*G99</f>
+        <f t="shared" si="6"/>
         <v>60</v>
       </c>
     </row>
@@ -5351,7 +5408,7 @@
         <v>0.03</v>
       </c>
       <c r="H100" s="5">
-        <f>F100*G100</f>
+        <f t="shared" si="6"/>
         <v>36</v>
       </c>
     </row>
@@ -5378,7 +5435,7 @@
         <v>0.03</v>
       </c>
       <c r="H101" s="5">
-        <f>F101*G101</f>
+        <f t="shared" si="6"/>
         <v>36</v>
       </c>
     </row>
@@ -5405,7 +5462,7 @@
         <v>0.05</v>
       </c>
       <c r="H102" s="5">
-        <f>F102*G102</f>
+        <f t="shared" si="6"/>
         <v>60</v>
       </c>
     </row>
@@ -5432,7 +5489,7 @@
         <v>1.8</v>
       </c>
       <c r="H103" s="5">
-        <f>F103*G103</f>
+        <f t="shared" si="6"/>
         <v>945</v>
       </c>
     </row>
@@ -5459,7 +5516,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="H104" s="5">
-        <f>F104*G104</f>
+        <f t="shared" si="6"/>
         <v>7.875</v>
       </c>
     </row>
@@ -5486,7 +5543,7 @@
         <v>0.25</v>
       </c>
       <c r="H105" s="5">
-        <f>F105*G105</f>
+        <f t="shared" si="6"/>
         <v>131.25</v>
       </c>
     </row>
@@ -5513,7 +5570,7 @@
         <v>0.125</v>
       </c>
       <c r="H106" s="5">
-        <f>F106*G106</f>
+        <f t="shared" si="6"/>
         <v>65.625</v>
       </c>
     </row>
@@ -5540,7 +5597,7 @@
         <v>0.25</v>
       </c>
       <c r="H107" s="5">
-        <f>F107*G107</f>
+        <f t="shared" si="6"/>
         <v>300</v>
       </c>
     </row>
@@ -5567,7 +5624,7 @@
         <v>0.5</v>
       </c>
       <c r="H108" s="5">
-        <f>F108*G108</f>
+        <f t="shared" si="6"/>
         <v>600</v>
       </c>
     </row>
@@ -5588,6 +5645,60 @@
       <c r="F109" s="5"/>
       <c r="G109" s="3"/>
       <c r="H109" s="5"/>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110" s="14">
+        <v>3112</v>
+      </c>
+      <c r="B110" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C110" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D110" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E110" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F110" s="16">
+        <v>785</v>
+      </c>
+      <c r="G110" s="11">
+        <v>0.125</v>
+      </c>
+      <c r="H110" s="16">
+        <f t="shared" si="6"/>
+        <v>98.125</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111" s="14">
+        <v>9647</v>
+      </c>
+      <c r="B111" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="C111" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="D111" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="E111" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="F111" s="16">
+        <v>1200</v>
+      </c>
+      <c r="G111" s="11">
+        <v>0.125</v>
+      </c>
+      <c r="H111" s="16">
+        <f t="shared" si="6"/>
+        <v>150</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:H88" xr:uid="{5D728A83-21A1-4AAF-B2FC-CCC59733812F}"/>

</xml_diff>